<commit_message>
chore: prepare database config and sync project updates
</commit_message>
<xml_diff>
--- a/outputs/blackwell_demo_v2/blackwell_technology_transmission_demo_v2.xlsx
+++ b/outputs/blackwell_demo_v2/blackwell_technology_transmission_demo_v2.xlsx
@@ -2,35 +2,31 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design_Principles" sheetId="1" r:id="R89bf3b60282d4289"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attribute_Audit" sheetId="2" r:id="Rbf8de301e6894553"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Property_Design_Guide" sheetId="3" r:id="R90579f5c98304873"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object_Instance_Index" sheetId="4" r:id="R7fc82ea7dd834bf5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_公司" sheetId="5" r:id="R57c495c0734b4906"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_GPU" sheetId="6" r:id="R409a342c162448cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_训练加速器" sheetId="7" r:id="Re5a891c5e09f4855"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_CPU" sheetId="8" r:id="R777382d1927b4376"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_互联技术" sheetId="9" r:id="R4e43dfd1dede4a84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_GPU架构世代" sheetId="10" r:id="Rf7d55d63338543ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_制程工艺" sheetId="11" r:id="R31332d83d4b4447c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_制程节点" sheetId="12" r:id="R586f4cef216e43fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_HBM" sheetId="13" r:id="R7ef180adc34c472b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_HBM世代" sheetId="14" r:id="R024f2f755af04d4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_封装技术世代" sheetId="15" r:id="R817c66fd6e9b487f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_先进封装技术" sheetId="16" r:id="Rfc88d4d964aa4fb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_封装方案" sheetId="17" r:id="Ra05ccd7be6904b87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_封装测试服务" sheetId="18" r:id="R75ff746a3f004311"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_后道工厂" sheetId="19" r:id="R9289e95c740e4a56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_ABF载板" sheetId="20" r:id="Re937e307bdae451a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_倒装键合机" sheetId="21" r:id="Rd5465a42a0654b4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_混合键合机" sheetId="22" r:id="Reeb58bdd34ea48d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_晶圆减薄机" sheetId="23" r:id="R5613794c26f9499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_资本开支" sheetId="24" r:id="Rf6fa995b87914432"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_数据中心计算应用" sheetId="25" r:id="R4609825ac02c41a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link_Type_Plan" sheetId="26" r:id="Rec1d7b3402414a55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link_Instance_Data" sheetId="27" r:id="Ree3642510ec9444f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Property_Evidence" sheetId="28" r:id="Raf61b7872f4f4f6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL_Import_Summary" sheetId="29" r:id="R8ac2df60b51f46d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design_Principles" sheetId="1" r:id="R16b7ac6a242c4d35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attribute_Audit" sheetId="2" r:id="R5d6b3360ce7b42e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Property_Design_Guide" sheetId="3" r:id="R62e0c872710049ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object_Instance_Index" sheetId="4" r:id="R712136e8764a4817"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_公司" sheetId="5" r:id="R4a535456b06a4eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_GPU" sheetId="6" r:id="R4b11b20fde40487a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_训练加速器" sheetId="7" r:id="R5d4bb566f7af4bfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_CPU" sheetId="8" r:id="Refc6e3c4bce04d8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_互联技术" sheetId="9" r:id="R6d4b71ad2c734467"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_GPU架构世代" sheetId="10" r:id="Rdea9cf05bf26452f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_制程工艺" sheetId="11" r:id="R20a4534429564ee3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_制程节点" sheetId="12" r:id="Rd56a9155eef8438c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_HBM" sheetId="13" r:id="R648398f81a254f91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_HBM世代" sheetId="14" r:id="Re8950d8d8049474f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_封装技术世代" sheetId="15" r:id="R07af75a032dc4a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_先进封装技术" sheetId="16" r:id="R2e35cdc8f23d48f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_封装方案" sheetId="17" r:id="R913fe41ab77a41cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_封装测试服务" sheetId="18" r:id="R726d2b4518fd43d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_后道工厂" sheetId="19" r:id="Rb40793b773ea4458"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_资本开支" sheetId="20" r:id="Re63595e8cc454bc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OT_数据中心计算应用" sheetId="21" r:id="R7b7b2968d79346eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link_Type_Plan" sheetId="22" r:id="R1d734d41ef184a2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link_Instance_Data" sheetId="23" r:id="Raf1ea30c66554c88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Property_Evidence" sheetId="24" r:id="Rcae4d139963f4e14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL_Import_Summary" sheetId="25" r:id="R71f6607d68f54ca3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1439,13 +1435,13 @@
         <x:v>ABF载板</x:v>
       </x:c>
       <x:c r="B12" s="17" t="str">
-        <x:v>supplier/target_application</x:v>
+        <x:v>AI加速器ABF载板等泛化实例和弱来源URL</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
-        <x:v>改为公司生产供给ABF载板、ABF载板供给于GPU</x:v>
+        <x:v>本版不导入ABF载板实例，也不导入ABF载板供给GPU或公司生产供给ABF载板关系；待有具体产品/产品族证据后再补</x:v>
       </x:c>
       <x:c r="D12" s="11" t="str">
-        <x:v>材料对象保留材料和需求驱动，供应链挂边。</x:v>
+        <x:v>避免把类别描述误当成真实实例。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -1453,13 +1449,13 @@
         <x:v>设备类OT</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>supplier</x:v>
+        <x:v>AI封装倒装键合机/先进封装混合键合机/HBM先进封装晶圆减薄机等泛化实例</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
-        <x:v>改为公司生产供给倒装键合机/混合键合机/晶圆减薄机</x:v>
+        <x:v>本版不导入倒装键合机、混合键合机、晶圆减薄机实例，也不导入相关公司供给或能力支撑关系；待有具体设备型号/产品系列证据后再补</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
-        <x:v>设备参数和设备供应商分开，便于查找设备瓶颈。</x:v>
+        <x:v>避免用泛化设备节点承载供应商关系，降低演示被追问的风险。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -1482,290 +1478,6 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="13.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="13.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="25.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="50.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="17.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="39.88999938964844" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="90.44000244140625" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>unique_id</x:v>
-      </x:c>
-      <x:c r="B1" s="14" t="str">
-        <x:v>name</x:v>
-      </x:c>
-      <x:c r="C1" s="14" t="str">
-        <x:v>name_en</x:v>
-      </x:c>
-      <x:c r="D1" s="14" t="str">
-        <x:v>object_type_name</x:v>
-      </x:c>
-      <x:c r="E1" s="14" t="str">
-        <x:v>description</x:v>
-      </x:c>
-      <x:c r="F1" s="14" t="str">
-        <x:v>dielectric_material</x:v>
-      </x:c>
-      <x:c r="G1" s="14" t="str">
-        <x:v>demand_driver</x:v>
-      </x:c>
-      <x:c r="H1" s="5" t="str">
-        <x:v>source_url</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="12" t="str">
-        <x:v>obj_abf_substrate</x:v>
-      </x:c>
-      <x:c r="B2" s="18" t="str">
-        <x:v>AI加速器ABF载板</x:v>
-      </x:c>
-      <x:c r="C2" s="18" t="str">
-        <x:v>ABF Substrate for AI Accelerators</x:v>
-      </x:c>
-      <x:c r="D2" s="18" t="str">
-        <x:v>ABF载板</x:v>
-      </x:c>
-      <x:c r="E2" s="18" t="str">
-        <x:v>Large-size ABF substrate used by high-end AI accelerator packages.</x:v>
-      </x:c>
-      <x:c r="F2" s="18" t="str">
-        <x:v>Ajinomoto build-up film</x:v>
-      </x:c>
-      <x:c r="G2" s="18" t="str">
-        <x:v>larger package size and advanced packaging demand</x:v>
-      </x:c>
-      <x:c r="H2" s="13" t="str">
-        <x:v>https://semiwiki.com/semiconductor-services/semiconductor-packaging/335318-understanding-tsmcs-cowos-l-packaging/</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="24.219999313354492" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="13.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="25.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="50.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="15.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="37.11000061035156" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="90.44000244140625" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>unique_id</x:v>
-      </x:c>
-      <x:c r="B1" s="14" t="str">
-        <x:v>name</x:v>
-      </x:c>
-      <x:c r="C1" s="14" t="str">
-        <x:v>name_en</x:v>
-      </x:c>
-      <x:c r="D1" s="14" t="str">
-        <x:v>object_type_name</x:v>
-      </x:c>
-      <x:c r="E1" s="14" t="str">
-        <x:v>description</x:v>
-      </x:c>
-      <x:c r="F1" s="14" t="str">
-        <x:v>equipment_category</x:v>
-      </x:c>
-      <x:c r="G1" s="14" t="str">
-        <x:v>supported_process</x:v>
-      </x:c>
-      <x:c r="H1" s="5" t="str">
-        <x:v>source_url</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="12" t="str">
-        <x:v>obj_equipment_flip_chip_bonder</x:v>
-      </x:c>
-      <x:c r="B2" s="18" t="str">
-        <x:v>AI封装倒装键合机</x:v>
-      </x:c>
-      <x:c r="C2" s="18" t="str">
-        <x:v>Flip-chip Bonder for AI Packaging</x:v>
-      </x:c>
-      <x:c r="D2" s="18" t="str">
-        <x:v>倒装键合机</x:v>
-      </x:c>
-      <x:c r="E2" s="18" t="str">
-        <x:v>Flip-chip bonding equipment used in advanced packaging assembly.</x:v>
-      </x:c>
-      <x:c r="F2" s="18" t="str">
-        <x:v>flip-chip bonding</x:v>
-      </x:c>
-      <x:c r="G2" s="18" t="str">
-        <x:v>die attach / chip placement for advanced package</x:v>
-      </x:c>
-      <x:c r="H2" s="13" t="str">
-        <x:v>https://semiwiki.com/semiconductor-services/semiconductor-packaging/335318-understanding-tsmcs-cowos-l-packaging/</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="22.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="15.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="29.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="51.220001220703125" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="15.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="90.44000244140625" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>unique_id</x:v>
-      </x:c>
-      <x:c r="B1" s="14" t="str">
-        <x:v>name</x:v>
-      </x:c>
-      <x:c r="C1" s="14" t="str">
-        <x:v>name_en</x:v>
-      </x:c>
-      <x:c r="D1" s="14" t="str">
-        <x:v>object_type_name</x:v>
-      </x:c>
-      <x:c r="E1" s="14" t="str">
-        <x:v>description</x:v>
-      </x:c>
-      <x:c r="F1" s="14" t="str">
-        <x:v>equipment_category</x:v>
-      </x:c>
-      <x:c r="G1" s="14" t="str">
-        <x:v>supported_process</x:v>
-      </x:c>
-      <x:c r="H1" s="5" t="str">
-        <x:v>source_url</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="12" t="str">
-        <x:v>obj_equipment_hybrid_bonder</x:v>
-      </x:c>
-      <x:c r="B2" s="18" t="str">
-        <x:v>先进封装混合键合机</x:v>
-      </x:c>
-      <x:c r="C2" s="18" t="str">
-        <x:v>Hybrid Bonder for Advanced Packaging</x:v>
-      </x:c>
-      <x:c r="D2" s="18" t="str">
-        <x:v>混合键合机</x:v>
-      </x:c>
-      <x:c r="E2" s="18" t="str">
-        <x:v>Hybrid bonding equipment relevant to advanced interconnect density.</x:v>
-      </x:c>
-      <x:c r="F2" s="18" t="str">
-        <x:v>hybrid bonding</x:v>
-      </x:c>
-      <x:c r="G2" s="18" t="str">
-        <x:v>wafer-to-wafer / die-to-wafer bonding</x:v>
-      </x:c>
-      <x:c r="H2" s="13" t="str">
-        <x:v>https://semiwiki.com/semiconductor-services/semiconductor-packaging/335318-understanding-tsmcs-cowos-l-packaging/</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="22.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="19.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="45.439998626708984" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="58.88999938964844" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="15.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="41.33000183105469" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="90.44000244140625" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>unique_id</x:v>
-      </x:c>
-      <x:c r="B1" s="14" t="str">
-        <x:v>name</x:v>
-      </x:c>
-      <x:c r="C1" s="14" t="str">
-        <x:v>name_en</x:v>
-      </x:c>
-      <x:c r="D1" s="14" t="str">
-        <x:v>object_type_name</x:v>
-      </x:c>
-      <x:c r="E1" s="14" t="str">
-        <x:v>description</x:v>
-      </x:c>
-      <x:c r="F1" s="14" t="str">
-        <x:v>equipment_category</x:v>
-      </x:c>
-      <x:c r="G1" s="14" t="str">
-        <x:v>supported_process</x:v>
-      </x:c>
-      <x:c r="H1" s="5" t="str">
-        <x:v>source_url</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="12" t="str">
-        <x:v>obj_equipment_wafer_thinning</x:v>
-      </x:c>
-      <x:c r="B2" s="18" t="str">
-        <x:v>HBM/先进封装晶圆减薄机</x:v>
-      </x:c>
-      <x:c r="C2" s="18" t="str">
-        <x:v>Wafer Thinning Equipment for HBM and Advanced Packaging</x:v>
-      </x:c>
-      <x:c r="D2" s="18" t="str">
-        <x:v>晶圆减薄机</x:v>
-      </x:c>
-      <x:c r="E2" s="18" t="str">
-        <x:v>Wafer thinning equipment used in HBM and advanced packaging process flows.</x:v>
-      </x:c>
-      <x:c r="F2" s="18" t="str">
-        <x:v>wafer thinning</x:v>
-      </x:c>
-      <x:c r="G2" s="18" t="str">
-        <x:v>backgrind / thinning for stacked memory and packaging</x:v>
-      </x:c>
-      <x:c r="H2" s="13" t="str">
-        <x:v>https://semiwiki.com/semiconductor-services/semiconductor-packaging/335318-understanding-tsmcs-cowos-l-packaging/</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1864,7 +1576,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1935,7 +1647,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2409,201 +2121,41 @@
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="10" t="str">
-        <x:v>lt_abf_substrate_supplies_to_graphics_processing_unit</x:v>
+        <x:v>lt_capital_expenditure_measures_for_assembly_test_service</x:v>
       </x:c>
       <x:c r="B24" s="17" t="str">
-        <x:v>ABF载板供给于GPU</x:v>
+        <x:v>资本开支统计对象封装测试服务</x:v>
       </x:c>
       <x:c r="C24" s="17" t="str">
-        <x:v>ABF载板</x:v>
+        <x:v>资本开支</x:v>
       </x:c>
       <x:c r="D24" s="17" t="str">
-        <x:v>GPU</x:v>
+        <x:v>封装测试服务</x:v>
       </x:c>
       <x:c r="E24" s="17" t="str">
-        <x:v>供给于</x:v>
+        <x:v>统计对象</x:v>
       </x:c>
       <x:c r="F24" s="11" t="str">
         <x:v>已有/确保存在</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
-      <x:c r="A25" s="10" t="str">
-        <x:v>lt_company_produces_for_abf_substrate</x:v>
-      </x:c>
-      <x:c r="B25" s="17" t="str">
-        <x:v>公司生产供给ABF载板</x:v>
-      </x:c>
-      <x:c r="C25" s="17" t="str">
-        <x:v>公司</x:v>
-      </x:c>
-      <x:c r="D25" s="17" t="str">
-        <x:v>ABF载板</x:v>
-      </x:c>
-      <x:c r="E25" s="17" t="str">
-        <x:v>生产供给</x:v>
-      </x:c>
-      <x:c r="F25" s="11" t="str">
-        <x:v>已有/确保存在</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="15" hidden="0" customHeight="1">
-      <x:c r="A26" s="10" t="str">
-        <x:v>lt_company_produces_for_flip_chip_bonding_equipment</x:v>
-      </x:c>
-      <x:c r="B26" s="17" t="str">
-        <x:v>公司生产供给倒装键合机</x:v>
-      </x:c>
-      <x:c r="C26" s="17" t="str">
-        <x:v>公司</x:v>
-      </x:c>
-      <x:c r="D26" s="17" t="str">
-        <x:v>倒装键合机</x:v>
-      </x:c>
-      <x:c r="E26" s="17" t="str">
-        <x:v>生产供给</x:v>
-      </x:c>
-      <x:c r="F26" s="11" t="str">
-        <x:v>新增/确保存在</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="15" hidden="0" customHeight="1">
-      <x:c r="A27" s="10" t="str">
-        <x:v>lt_company_produces_for_hybrid_bonding_equipment</x:v>
-      </x:c>
-      <x:c r="B27" s="17" t="str">
-        <x:v>公司生产供给混合键合机</x:v>
-      </x:c>
-      <x:c r="C27" s="17" t="str">
-        <x:v>公司</x:v>
-      </x:c>
-      <x:c r="D27" s="17" t="str">
-        <x:v>混合键合机</x:v>
-      </x:c>
-      <x:c r="E27" s="17" t="str">
-        <x:v>生产供给</x:v>
-      </x:c>
-      <x:c r="F27" s="11" t="str">
-        <x:v>新增/确保存在</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="15" hidden="0" customHeight="1">
-      <x:c r="A28" s="10" t="str">
-        <x:v>lt_company_produces_for_wafer_thinning_equipment</x:v>
-      </x:c>
-      <x:c r="B28" s="17" t="str">
-        <x:v>公司生产供给晶圆减薄机</x:v>
-      </x:c>
-      <x:c r="C28" s="17" t="str">
-        <x:v>公司</x:v>
-      </x:c>
-      <x:c r="D28" s="17" t="str">
-        <x:v>晶圆减薄机</x:v>
-      </x:c>
-      <x:c r="E28" s="17" t="str">
-        <x:v>生产供给</x:v>
-      </x:c>
-      <x:c r="F28" s="11" t="str">
-        <x:v>新增/确保存在</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="15" hidden="0" customHeight="1">
-      <x:c r="A29" s="10" t="str">
-        <x:v>lt_flip_chip_bonding_equipment_supports_capability_of_assembly_test_service</x:v>
-      </x:c>
-      <x:c r="B29" s="17" t="str">
-        <x:v>倒装键合机能力支撑封装测试服务</x:v>
-      </x:c>
-      <x:c r="C29" s="17" t="str">
-        <x:v>倒装键合机</x:v>
-      </x:c>
-      <x:c r="D29" s="17" t="str">
-        <x:v>封装测试服务</x:v>
-      </x:c>
-      <x:c r="E29" s="17" t="str">
-        <x:v>能力支撑</x:v>
-      </x:c>
-      <x:c r="F29" s="11" t="str">
-        <x:v>已有/确保存在</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="15" hidden="0" customHeight="1">
-      <x:c r="A30" s="10" t="str">
-        <x:v>lt_hybrid_bonding_equipment_supports_capability_of_assembly_test_service</x:v>
-      </x:c>
-      <x:c r="B30" s="17" t="str">
-        <x:v>混合键合机能力支撑封装测试服务</x:v>
-      </x:c>
-      <x:c r="C30" s="17" t="str">
-        <x:v>混合键合机</x:v>
-      </x:c>
-      <x:c r="D30" s="17" t="str">
-        <x:v>封装测试服务</x:v>
-      </x:c>
-      <x:c r="E30" s="17" t="str">
-        <x:v>能力支撑</x:v>
-      </x:c>
-      <x:c r="F30" s="11" t="str">
-        <x:v>已有/确保存在</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="15" hidden="0" customHeight="1">
-      <x:c r="A31" s="10" t="str">
-        <x:v>lt_wafer_thinning_equipment_supports_capability_of_assembly_test_service</x:v>
-      </x:c>
-      <x:c r="B31" s="17" t="str">
-        <x:v>晶圆减薄机能力支撑封装测试服务</x:v>
-      </x:c>
-      <x:c r="C31" s="17" t="str">
-        <x:v>晶圆减薄机</x:v>
-      </x:c>
-      <x:c r="D31" s="17" t="str">
-        <x:v>封装测试服务</x:v>
-      </x:c>
-      <x:c r="E31" s="17" t="str">
-        <x:v>能力支撑</x:v>
-      </x:c>
-      <x:c r="F31" s="11" t="str">
-        <x:v>已有/确保存在</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="15" hidden="0" customHeight="1">
-      <x:c r="A32" s="10" t="str">
-        <x:v>lt_capital_expenditure_measures_for_assembly_test_service</x:v>
-      </x:c>
-      <x:c r="B32" s="17" t="str">
-        <x:v>资本开支统计对象封装测试服务</x:v>
-      </x:c>
-      <x:c r="C32" s="17" t="str">
+      <x:c r="A25" s="12" t="str">
+        <x:v>lt_capital_expenditure_measures_for_backend_facility</x:v>
+      </x:c>
+      <x:c r="B25" s="18" t="str">
+        <x:v>资本开支统计对象后道工厂</x:v>
+      </x:c>
+      <x:c r="C25" s="18" t="str">
         <x:v>资本开支</x:v>
       </x:c>
-      <x:c r="D32" s="17" t="str">
-        <x:v>封装测试服务</x:v>
-      </x:c>
-      <x:c r="E32" s="17" t="str">
+      <x:c r="D25" s="18" t="str">
+        <x:v>后道工厂</x:v>
+      </x:c>
+      <x:c r="E25" s="18" t="str">
         <x:v>统计对象</x:v>
       </x:c>
-      <x:c r="F32" s="11" t="str">
-        <x:v>已有/确保存在</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="15" hidden="0" customHeight="1">
-      <x:c r="A33" s="12" t="str">
-        <x:v>lt_capital_expenditure_measures_for_backend_facility</x:v>
-      </x:c>
-      <x:c r="B33" s="18" t="str">
-        <x:v>资本开支统计对象后道工厂</x:v>
-      </x:c>
-      <x:c r="C33" s="18" t="str">
-        <x:v>资本开支</x:v>
-      </x:c>
-      <x:c r="D33" s="18" t="str">
-        <x:v>后道工厂</x:v>
-      </x:c>
-      <x:c r="E33" s="18" t="str">
-        <x:v>统计对象</x:v>
-      </x:c>
-      <x:c r="F33" s="13" t="str">
+      <x:c r="F25" s="13" t="str">
         <x:v>已有/确保存在</x:v>
       </x:c>
     </x:row>
@@ -2612,7 +2164,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3101,256 +2653,35 @@
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="10" t="str">
-        <x:v>link_abf_to_b200</x:v>
+        <x:v>link_capex_to_service</x:v>
       </x:c>
       <x:c r="B29" s="17" t="str">
-        <x:v>lt_abf_substrate_supplies_to_graphics_processing_unit</x:v>
+        <x:v>lt_capital_expenditure_measures_for_assembly_test_service</x:v>
       </x:c>
       <x:c r="C29" s="17" t="str">
-        <x:v>obj_abf_substrate</x:v>
+        <x:v>obj_metric_tsmc_adv_packaging_capex</x:v>
       </x:c>
       <x:c r="D29" s="17" t="str">
-        <x:v>obj_gpu_nvidia_b200</x:v>
+        <x:v>obj_service_tsmc_cowos</x:v>
       </x:c>
       <x:c r="E29" s="11" t="str">
-        <x:v>Large ABF substrates supply high-end AI accelerator packages.</x:v>
+        <x:v>Capex is measured against packaging service capacity.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
-      <x:c r="A30" s="10" t="str">
-        <x:v>link_ibiden_to_abf</x:v>
-      </x:c>
-      <x:c r="B30" s="17" t="str">
-        <x:v>lt_company_produces_for_abf_substrate</x:v>
-      </x:c>
-      <x:c r="C30" s="17" t="str">
-        <x:v>obj_company_ibiden</x:v>
-      </x:c>
-      <x:c r="D30" s="17" t="str">
-        <x:v>obj_abf_substrate</x:v>
-      </x:c>
-      <x:c r="E30" s="11" t="str">
-        <x:v>ABF supplier relationship.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="15" hidden="0" customHeight="1">
-      <x:c r="A31" s="10" t="str">
-        <x:v>link_unimicron_to_abf</x:v>
-      </x:c>
-      <x:c r="B31" s="17" t="str">
-        <x:v>lt_company_produces_for_abf_substrate</x:v>
-      </x:c>
-      <x:c r="C31" s="17" t="str">
-        <x:v>obj_company_unimicron</x:v>
-      </x:c>
-      <x:c r="D31" s="17" t="str">
-        <x:v>obj_abf_substrate</x:v>
-      </x:c>
-      <x:c r="E31" s="11" t="str">
-        <x:v>ABF supplier relationship.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="15" hidden="0" customHeight="1">
-      <x:c r="A32" s="10" t="str">
-        <x:v>link_shinko_to_abf</x:v>
-      </x:c>
-      <x:c r="B32" s="17" t="str">
-        <x:v>lt_company_produces_for_abf_substrate</x:v>
-      </x:c>
-      <x:c r="C32" s="17" t="str">
-        <x:v>obj_company_shinko</x:v>
-      </x:c>
-      <x:c r="D32" s="17" t="str">
-        <x:v>obj_abf_substrate</x:v>
-      </x:c>
-      <x:c r="E32" s="11" t="str">
-        <x:v>ABF supplier relationship.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="15" hidden="0" customHeight="1">
-      <x:c r="A33" s="10" t="str">
-        <x:v>link_besi_to_flip_chip</x:v>
-      </x:c>
-      <x:c r="B33" s="17" t="str">
-        <x:v>lt_company_produces_for_flip_chip_bonding_equipment</x:v>
-      </x:c>
-      <x:c r="C33" s="17" t="str">
-        <x:v>obj_company_besi</x:v>
-      </x:c>
-      <x:c r="D33" s="17" t="str">
-        <x:v>obj_equipment_flip_chip_bonder</x:v>
-      </x:c>
-      <x:c r="E33" s="11" t="str">
-        <x:v>Equipment supplier relationship.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="15" hidden="0" customHeight="1">
-      <x:c r="A34" s="10" t="str">
-        <x:v>link_asmpt_to_flip_chip</x:v>
-      </x:c>
-      <x:c r="B34" s="17" t="str">
-        <x:v>lt_company_produces_for_flip_chip_bonding_equipment</x:v>
-      </x:c>
-      <x:c r="C34" s="17" t="str">
-        <x:v>obj_company_asmpt</x:v>
-      </x:c>
-      <x:c r="D34" s="17" t="str">
-        <x:v>obj_equipment_flip_chip_bonder</x:v>
-      </x:c>
-      <x:c r="E34" s="11" t="str">
-        <x:v>Equipment supplier relationship.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="15" hidden="0" customHeight="1">
-      <x:c r="A35" s="10" t="str">
-        <x:v>link_kulicke_to_flip_chip</x:v>
-      </x:c>
-      <x:c r="B35" s="17" t="str">
-        <x:v>lt_company_produces_for_flip_chip_bonding_equipment</x:v>
-      </x:c>
-      <x:c r="C35" s="17" t="str">
-        <x:v>obj_company_kulicke_soffa</x:v>
-      </x:c>
-      <x:c r="D35" s="17" t="str">
-        <x:v>obj_equipment_flip_chip_bonder</x:v>
-      </x:c>
-      <x:c r="E35" s="11" t="str">
-        <x:v>Equipment supplier relationship.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="15" hidden="0" customHeight="1">
-      <x:c r="A36" s="10" t="str">
-        <x:v>link_besi_to_hybrid</x:v>
-      </x:c>
-      <x:c r="B36" s="17" t="str">
-        <x:v>lt_company_produces_for_hybrid_bonding_equipment</x:v>
-      </x:c>
-      <x:c r="C36" s="17" t="str">
-        <x:v>obj_company_besi</x:v>
-      </x:c>
-      <x:c r="D36" s="17" t="str">
-        <x:v>obj_equipment_hybrid_bonder</x:v>
-      </x:c>
-      <x:c r="E36" s="11" t="str">
-        <x:v>Equipment supplier relationship.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="15" hidden="0" customHeight="1">
-      <x:c r="A37" s="10" t="str">
-        <x:v>link_asmpt_to_hybrid</x:v>
-      </x:c>
-      <x:c r="B37" s="17" t="str">
-        <x:v>lt_company_produces_for_hybrid_bonding_equipment</x:v>
-      </x:c>
-      <x:c r="C37" s="17" t="str">
-        <x:v>obj_company_asmpt</x:v>
-      </x:c>
-      <x:c r="D37" s="17" t="str">
-        <x:v>obj_equipment_hybrid_bonder</x:v>
-      </x:c>
-      <x:c r="E37" s="11" t="str">
-        <x:v>Equipment supplier relationship.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="15" hidden="0" customHeight="1">
-      <x:c r="A38" s="10" t="str">
-        <x:v>link_disco_to_thinning</x:v>
-      </x:c>
-      <x:c r="B38" s="17" t="str">
-        <x:v>lt_company_produces_for_wafer_thinning_equipment</x:v>
-      </x:c>
-      <x:c r="C38" s="17" t="str">
-        <x:v>obj_company_disco</x:v>
-      </x:c>
-      <x:c r="D38" s="17" t="str">
-        <x:v>obj_equipment_wafer_thinning</x:v>
-      </x:c>
-      <x:c r="E38" s="11" t="str">
-        <x:v>Equipment supplier relationship.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="15" hidden="0" customHeight="1">
-      <x:c r="A39" s="10" t="str">
-        <x:v>link_flip_chip_to_service</x:v>
-      </x:c>
-      <x:c r="B39" s="17" t="str">
-        <x:v>lt_flip_chip_bonding_equipment_supports_capability_of_assembly_test_service</x:v>
-      </x:c>
-      <x:c r="C39" s="17" t="str">
-        <x:v>obj_equipment_flip_chip_bonder</x:v>
-      </x:c>
-      <x:c r="D39" s="17" t="str">
-        <x:v>obj_service_tsmc_cowos</x:v>
-      </x:c>
-      <x:c r="E39" s="11" t="str">
-        <x:v>Flip-chip bonding equipment supports advanced packaging service.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="15" hidden="0" customHeight="1">
-      <x:c r="A40" s="10" t="str">
-        <x:v>link_hybrid_to_service</x:v>
-      </x:c>
-      <x:c r="B40" s="17" t="str">
-        <x:v>lt_hybrid_bonding_equipment_supports_capability_of_assembly_test_service</x:v>
-      </x:c>
-      <x:c r="C40" s="17" t="str">
-        <x:v>obj_equipment_hybrid_bonder</x:v>
-      </x:c>
-      <x:c r="D40" s="17" t="str">
-        <x:v>obj_service_tsmc_cowos</x:v>
-      </x:c>
-      <x:c r="E40" s="11" t="str">
-        <x:v>Hybrid bonding equipment supports advanced packaging service.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="15" hidden="0" customHeight="1">
-      <x:c r="A41" s="10" t="str">
-        <x:v>link_thinning_to_service</x:v>
-      </x:c>
-      <x:c r="B41" s="17" t="str">
-        <x:v>lt_wafer_thinning_equipment_supports_capability_of_assembly_test_service</x:v>
-      </x:c>
-      <x:c r="C41" s="17" t="str">
-        <x:v>obj_equipment_wafer_thinning</x:v>
-      </x:c>
-      <x:c r="D41" s="17" t="str">
-        <x:v>obj_service_tsmc_cowos</x:v>
-      </x:c>
-      <x:c r="E41" s="11" t="str">
-        <x:v>Wafer thinning equipment supports advanced packaging and HBM process flows.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="15" hidden="0" customHeight="1">
-      <x:c r="A42" s="10" t="str">
-        <x:v>link_capex_to_service</x:v>
-      </x:c>
-      <x:c r="B42" s="17" t="str">
-        <x:v>lt_capital_expenditure_measures_for_assembly_test_service</x:v>
-      </x:c>
-      <x:c r="C42" s="17" t="str">
+      <x:c r="A30" s="12" t="str">
+        <x:v>link_capex_to_facility</x:v>
+      </x:c>
+      <x:c r="B30" s="18" t="str">
+        <x:v>lt_capital_expenditure_measures_for_backend_facility</x:v>
+      </x:c>
+      <x:c r="C30" s="18" t="str">
         <x:v>obj_metric_tsmc_adv_packaging_capex</x:v>
       </x:c>
-      <x:c r="D42" s="17" t="str">
-        <x:v>obj_service_tsmc_cowos</x:v>
-      </x:c>
-      <x:c r="E42" s="11" t="str">
-        <x:v>Capex is measured against packaging service capacity.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="15" hidden="0" customHeight="1">
-      <x:c r="A43" s="12" t="str">
-        <x:v>link_capex_to_facility</x:v>
-      </x:c>
-      <x:c r="B43" s="18" t="str">
-        <x:v>lt_capital_expenditure_measures_for_backend_facility</x:v>
-      </x:c>
-      <x:c r="C43" s="18" t="str">
-        <x:v>obj_metric_tsmc_adv_packaging_capex</x:v>
-      </x:c>
-      <x:c r="D43" s="18" t="str">
+      <x:c r="D30" s="18" t="str">
         <x:v>obj_facility_tsmc_ap6</x:v>
       </x:c>
-      <x:c r="E43" s="13" t="str">
+      <x:c r="E30" s="13" t="str">
         <x:v>Capex is measured against backend facility expansion.</x:v>
       </x:c>
     </x:row>
@@ -3359,7 +2690,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3917,7 +3248,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3946,7 +3277,7 @@
         <x:v>instance_tables</x:v>
       </x:c>
       <x:c r="B3" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -3954,7 +3285,7 @@
         <x:v>object_instances</x:v>
       </x:c>
       <x:c r="B4" s="11" t="n">
-        <x:v>35</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -3962,7 +3293,7 @@
         <x:v>link_types_ensured</x:v>
       </x:c>
       <x:c r="B5" s="11" t="n">
-        <x:v>32</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -3970,7 +3301,7 @@
         <x:v>link_instances</x:v>
       </x:c>
       <x:c r="B6" s="11" t="n">
-        <x:v>42</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -4189,421 +3520,267 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="10" t="str">
-        <x:v>obj_company_ibiden</x:v>
+        <x:v>obj_gpu_nvidia_b200</x:v>
       </x:c>
       <x:c r="B7" s="17" t="str">
-        <x:v>揖斐电</x:v>
+        <x:v>NVIDIA B200 Tensor Core GPU</x:v>
       </x:c>
       <x:c r="C7" s="17" t="str">
-        <x:v>公司</x:v>
+        <x:v>GPU</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
-        <x:v>ABF substrate supplier.</x:v>
+        <x:v>Blackwell-generation Tensor Core GPU used in GB200 Grace Blackwell Superchip and HGX B200 platforms.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="10" t="str">
-        <x:v>obj_company_unimicron</x:v>
+        <x:v>obj_training_accelerator_gb200</x:v>
       </x:c>
       <x:c r="B8" s="17" t="str">
-        <x:v>欣兴电子</x:v>
+        <x:v>NVIDIA GB200 Grace Blackwell Superchip</x:v>
       </x:c>
       <x:c r="C8" s="17" t="str">
-        <x:v>公司</x:v>
+        <x:v>训练加速器</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
-        <x:v>ABF substrate supplier.</x:v>
+        <x:v>Training accelerator module combining one Grace CPU and two Blackwell GPUs.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="10" t="str">
-        <x:v>obj_company_shinko</x:v>
+        <x:v>obj_cpu_nvidia_grace</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>新光电气</x:v>
+        <x:v>NVIDIA Grace CPU</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
-        <x:v>公司</x:v>
+        <x:v>CPU</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
-        <x:v>ABF substrate supplier.</x:v>
+        <x:v>CPU used with Blackwell GPUs in the GB200 Grace Blackwell Superchip.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="10" t="str">
-        <x:v>obj_company_besi</x:v>
+        <x:v>obj_interconnect_nvlink</x:v>
       </x:c>
       <x:c r="B10" s="17" t="str">
-        <x:v>BESI</x:v>
+        <x:v>NVIDIA NVLink</x:v>
       </x:c>
       <x:c r="C10" s="17" t="str">
-        <x:v>公司</x:v>
+        <x:v>互联技术</x:v>
       </x:c>
       <x:c r="D10" s="11" t="str">
-        <x:v>Advanced bonding equipment supplier.</x:v>
+        <x:v>High-speed interconnect technology used by NVIDIA AI accelerator platforms.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="10" t="str">
-        <x:v>obj_company_asmpt</x:v>
+        <x:v>obj_interconnect_nvlink_c2c</x:v>
       </x:c>
       <x:c r="B11" s="17" t="str">
-        <x:v>ASMPT</x:v>
+        <x:v>NVIDIA NVLink-C2C</x:v>
       </x:c>
       <x:c r="C11" s="17" t="str">
-        <x:v>公司</x:v>
+        <x:v>互联技术</x:v>
       </x:c>
       <x:c r="D11" s="11" t="str">
-        <x:v>Advanced bonding equipment supplier.</x:v>
+        <x:v>Chip-to-chip interconnect technology used between Grace CPU and Blackwell GPUs.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="10" t="str">
-        <x:v>obj_company_kulicke_soffa</x:v>
+        <x:v>obj_gpu_arch_blackwell</x:v>
       </x:c>
       <x:c r="B12" s="17" t="str">
-        <x:v>K&amp;S</x:v>
+        <x:v>NVIDIA Blackwell架构</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
-        <x:v>公司</x:v>
+        <x:v>GPU架构世代</x:v>
       </x:c>
       <x:c r="D12" s="11" t="str">
-        <x:v>Bonding equipment supplier.</x:v>
+        <x:v>GPU architecture generation centered on AI training and inference scaling.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="10" t="str">
-        <x:v>obj_company_disco</x:v>
+        <x:v>obj_process_platform_tsmc_4np</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>DISCO</x:v>
+        <x:v>TSMC 4NP</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
-        <x:v>公司</x:v>
+        <x:v>制程工艺</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
-        <x:v>Wafer thinning and dicing equipment supplier.</x:v>
+        <x:v>Custom-built TSMC process disclosed by NVIDIA for Blackwell-architecture GPUs; scope is expressed through GPU and architecture link instances.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="10" t="str">
-        <x:v>obj_gpu_nvidia_b200</x:v>
+        <x:v>obj_process_node_4nm_class</x:v>
       </x:c>
       <x:c r="B14" s="17" t="str">
-        <x:v>NVIDIA B200 Tensor Core GPU</x:v>
+        <x:v>4nm-class制程节点</x:v>
       </x:c>
       <x:c r="C14" s="17" t="str">
-        <x:v>GPU</x:v>
+        <x:v>制程节点</x:v>
       </x:c>
       <x:c r="D14" s="11" t="str">
-        <x:v>Blackwell-generation Tensor Core GPU used in GB200 Grace Blackwell Superchip and HGX B200 platforms.</x:v>
+        <x:v>Industry node class used to group TSMC 4nm-class process variants; not a literal physical feature size.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="10" t="str">
-        <x:v>obj_training_accelerator_gb200</x:v>
+        <x:v>obj_hbm_skhynix_hbm3e</x:v>
       </x:c>
       <x:c r="B15" s="17" t="str">
-        <x:v>NVIDIA GB200 Grace Blackwell Superchip</x:v>
+        <x:v>SK海力士HBM3E 12Hi</x:v>
       </x:c>
       <x:c r="C15" s="17" t="str">
-        <x:v>训练加速器</x:v>
+        <x:v>HBM</x:v>
       </x:c>
       <x:c r="D15" s="11" t="str">
-        <x:v>Training accelerator module combining one Grace CPU and two Blackwell GPUs.</x:v>
+        <x:v>12-high HBM3E product relevant to AI accelerator memory capacity growth.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="10" t="str">
-        <x:v>obj_cpu_nvidia_grace</x:v>
+        <x:v>obj_hbm_micron_hbm3e</x:v>
       </x:c>
       <x:c r="B16" s="17" t="str">
-        <x:v>NVIDIA Grace CPU</x:v>
+        <x:v>美光HBM3E 24GB</x:v>
       </x:c>
       <x:c r="C16" s="17" t="str">
-        <x:v>CPU</x:v>
+        <x:v>HBM</x:v>
       </x:c>
       <x:c r="D16" s="11" t="str">
-        <x:v>CPU used with Blackwell GPUs in the GB200 Grace Blackwell Superchip.</x:v>
+        <x:v>24GB HBM3E product relevant to AI accelerator memory bandwidth.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="10" t="str">
-        <x:v>obj_interconnect_nvlink</x:v>
+        <x:v>obj_hbm_samsung_hbm3e</x:v>
       </x:c>
       <x:c r="B17" s="17" t="str">
-        <x:v>NVIDIA NVLink</x:v>
+        <x:v>三星HBM3E</x:v>
       </x:c>
       <x:c r="C17" s="17" t="str">
-        <x:v>互联技术</x:v>
+        <x:v>HBM</x:v>
       </x:c>
       <x:c r="D17" s="11" t="str">
-        <x:v>High-speed interconnect technology used by NVIDIA AI accelerator platforms.</x:v>
+        <x:v>Samsung HBM3E product family.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="10" t="str">
-        <x:v>obj_interconnect_nvlink_c2c</x:v>
+        <x:v>obj_hbm_generation_hbm3e</x:v>
       </x:c>
       <x:c r="B18" s="17" t="str">
-        <x:v>NVIDIA NVLink-C2C</x:v>
+        <x:v>HBM3E世代</x:v>
       </x:c>
       <x:c r="C18" s="17" t="str">
-        <x:v>互联技术</x:v>
+        <x:v>HBM世代</x:v>
       </x:c>
       <x:c r="D18" s="11" t="str">
-        <x:v>Chip-to-chip interconnect technology used between Grace CPU and Blackwell GPUs.</x:v>
+        <x:v>Enhanced HBM3 generation used in advanced AI accelerator products.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="10" t="str">
-        <x:v>obj_gpu_arch_blackwell</x:v>
+        <x:v>obj_packaging_generation_2_5d</x:v>
       </x:c>
       <x:c r="B19" s="17" t="str">
-        <x:v>NVIDIA Blackwell架构</x:v>
+        <x:v>2.5D先进封装</x:v>
       </x:c>
       <x:c r="C19" s="17" t="str">
-        <x:v>GPU架构世代</x:v>
+        <x:v>封装技术世代</x:v>
       </x:c>
       <x:c r="D19" s="11" t="str">
-        <x:v>GPU architecture generation centered on AI training and inference scaling.</x:v>
+        <x:v>Advanced packaging class represented by interposer, RDL or substrate-based multi-die integration.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="10" t="str">
-        <x:v>obj_process_platform_tsmc_4np</x:v>
+        <x:v>obj_advanced_packaging_cowos</x:v>
       </x:c>
       <x:c r="B20" s="17" t="str">
-        <x:v>TSMC 4NP</x:v>
+        <x:v>CoWoS</x:v>
       </x:c>
       <x:c r="C20" s="17" t="str">
-        <x:v>制程工艺</x:v>
+        <x:v>先进封装技术</x:v>
       </x:c>
       <x:c r="D20" s="11" t="str">
-        <x:v>Custom-built TSMC process disclosed by NVIDIA for Blackwell-architecture GPUs; scope is expressed through GPU and architecture link instances.</x:v>
+        <x:v>Chip-on-wafer-on-substrate advanced packaging technology platform for high-end AI accelerators.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="10" t="str">
-        <x:v>obj_process_node_4nm_class</x:v>
+        <x:v>obj_packaging_solution_tsmc_cowos_l</x:v>
       </x:c>
       <x:c r="B21" s="17" t="str">
-        <x:v>4nm-class制程节点</x:v>
+        <x:v>TSMC CoWoS-L</x:v>
       </x:c>
       <x:c r="C21" s="17" t="str">
-        <x:v>制程节点</x:v>
+        <x:v>封装方案</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
-        <x:v>Industry node class used to group TSMC 4nm-class process variants; not a literal physical feature size.</x:v>
+        <x:v>Concrete CoWoS solution variant using local silicon interconnect bridges for large multi-die AI packages.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="10" t="str">
-        <x:v>obj_hbm_skhynix_hbm3e</x:v>
+        <x:v>obj_service_tsmc_cowos</x:v>
       </x:c>
       <x:c r="B22" s="17" t="str">
-        <x:v>SK海力士HBM3E 12Hi</x:v>
+        <x:v>台积电CoWoS封装测试服务</x:v>
       </x:c>
       <x:c r="C22" s="17" t="str">
-        <x:v>HBM</x:v>
+        <x:v>封装测试服务</x:v>
       </x:c>
       <x:c r="D22" s="11" t="str">
-        <x:v>12-high HBM3E product relevant to AI accelerator memory capacity growth.</x:v>
+        <x:v>Commercial packaging and testing service capacity required to manufacture CoWoS-based AI accelerator products.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="10" t="str">
-        <x:v>obj_hbm_micron_hbm3e</x:v>
+        <x:v>obj_facility_tsmc_ap6</x:v>
       </x:c>
       <x:c r="B23" s="17" t="str">
-        <x:v>美光HBM3E 24GB</x:v>
+        <x:v>台积电CoWoS后道产能</x:v>
       </x:c>
       <x:c r="C23" s="17" t="str">
-        <x:v>HBM</x:v>
+        <x:v>后道工厂</x:v>
       </x:c>
       <x:c r="D23" s="11" t="str">
-        <x:v>24GB HBM3E product relevant to AI accelerator memory bandwidth.</x:v>
+        <x:v>TSMC backend capacity associated with CoWoS advanced packaging expansion.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="10" t="str">
-        <x:v>obj_hbm_samsung_hbm3e</x:v>
+        <x:v>obj_metric_tsmc_adv_packaging_capex</x:v>
       </x:c>
       <x:c r="B24" s="17" t="str">
-        <x:v>三星HBM3E</x:v>
+        <x:v>台积电先进封装扩产资本开支</x:v>
       </x:c>
       <x:c r="C24" s="17" t="str">
-        <x:v>HBM</x:v>
+        <x:v>资本开支</x:v>
       </x:c>
       <x:c r="D24" s="11" t="str">
-        <x:v>Samsung HBM3E product family.</x:v>
+        <x:v>Capital expenditure associated with advanced packaging and CoWoS capacity expansion.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
-      <x:c r="A25" s="10" t="str">
-        <x:v>obj_hbm_generation_hbm3e</x:v>
-      </x:c>
-      <x:c r="B25" s="17" t="str">
-        <x:v>HBM3E世代</x:v>
-      </x:c>
-      <x:c r="C25" s="17" t="str">
-        <x:v>HBM世代</x:v>
-      </x:c>
-      <x:c r="D25" s="11" t="str">
-        <x:v>Enhanced HBM3 generation used in advanced AI accelerator products.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="15" hidden="0" customHeight="1">
-      <x:c r="A26" s="10" t="str">
-        <x:v>obj_packaging_generation_2_5d</x:v>
-      </x:c>
-      <x:c r="B26" s="17" t="str">
-        <x:v>2.5D先进封装</x:v>
-      </x:c>
-      <x:c r="C26" s="17" t="str">
-        <x:v>封装技术世代</x:v>
-      </x:c>
-      <x:c r="D26" s="11" t="str">
-        <x:v>Advanced packaging class represented by interposer, RDL or substrate-based multi-die integration.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="15" hidden="0" customHeight="1">
-      <x:c r="A27" s="10" t="str">
-        <x:v>obj_advanced_packaging_cowos</x:v>
-      </x:c>
-      <x:c r="B27" s="17" t="str">
-        <x:v>CoWoS</x:v>
-      </x:c>
-      <x:c r="C27" s="17" t="str">
-        <x:v>先进封装技术</x:v>
-      </x:c>
-      <x:c r="D27" s="11" t="str">
-        <x:v>Chip-on-wafer-on-substrate advanced packaging technology platform for high-end AI accelerators.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="15" hidden="0" customHeight="1">
-      <x:c r="A28" s="10" t="str">
-        <x:v>obj_packaging_solution_tsmc_cowos_l</x:v>
-      </x:c>
-      <x:c r="B28" s="17" t="str">
-        <x:v>TSMC CoWoS-L</x:v>
-      </x:c>
-      <x:c r="C28" s="17" t="str">
-        <x:v>封装方案</x:v>
-      </x:c>
-      <x:c r="D28" s="11" t="str">
-        <x:v>Concrete CoWoS solution variant using local silicon interconnect bridges for large multi-die AI packages.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="15" hidden="0" customHeight="1">
-      <x:c r="A29" s="10" t="str">
-        <x:v>obj_service_tsmc_cowos</x:v>
-      </x:c>
-      <x:c r="B29" s="17" t="str">
-        <x:v>台积电CoWoS封装测试服务</x:v>
-      </x:c>
-      <x:c r="C29" s="17" t="str">
-        <x:v>封装测试服务</x:v>
-      </x:c>
-      <x:c r="D29" s="11" t="str">
-        <x:v>Commercial packaging and testing service capacity required to manufacture CoWoS-based AI accelerator products.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="15" hidden="0" customHeight="1">
-      <x:c r="A30" s="10" t="str">
-        <x:v>obj_facility_tsmc_ap6</x:v>
-      </x:c>
-      <x:c r="B30" s="17" t="str">
-        <x:v>台积电CoWoS后道产能</x:v>
-      </x:c>
-      <x:c r="C30" s="17" t="str">
-        <x:v>后道工厂</x:v>
-      </x:c>
-      <x:c r="D30" s="11" t="str">
-        <x:v>TSMC backend capacity associated with CoWoS advanced packaging expansion.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="15" hidden="0" customHeight="1">
-      <x:c r="A31" s="10" t="str">
-        <x:v>obj_abf_substrate</x:v>
-      </x:c>
-      <x:c r="B31" s="17" t="str">
-        <x:v>AI加速器ABF载板</x:v>
-      </x:c>
-      <x:c r="C31" s="17" t="str">
-        <x:v>ABF载板</x:v>
-      </x:c>
-      <x:c r="D31" s="11" t="str">
-        <x:v>Large-size ABF substrate used by high-end AI accelerator packages.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="15" hidden="0" customHeight="1">
-      <x:c r="A32" s="10" t="str">
-        <x:v>obj_equipment_flip_chip_bonder</x:v>
-      </x:c>
-      <x:c r="B32" s="17" t="str">
-        <x:v>AI封装倒装键合机</x:v>
-      </x:c>
-      <x:c r="C32" s="17" t="str">
-        <x:v>倒装键合机</x:v>
-      </x:c>
-      <x:c r="D32" s="11" t="str">
-        <x:v>Flip-chip bonding equipment used in advanced packaging assembly.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="15" hidden="0" customHeight="1">
-      <x:c r="A33" s="10" t="str">
-        <x:v>obj_equipment_hybrid_bonder</x:v>
-      </x:c>
-      <x:c r="B33" s="17" t="str">
-        <x:v>先进封装混合键合机</x:v>
-      </x:c>
-      <x:c r="C33" s="17" t="str">
-        <x:v>混合键合机</x:v>
-      </x:c>
-      <x:c r="D33" s="11" t="str">
-        <x:v>Hybrid bonding equipment relevant to advanced interconnect density.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="15" hidden="0" customHeight="1">
-      <x:c r="A34" s="10" t="str">
-        <x:v>obj_equipment_wafer_thinning</x:v>
-      </x:c>
-      <x:c r="B34" s="17" t="str">
-        <x:v>HBM/先进封装晶圆减薄机</x:v>
-      </x:c>
-      <x:c r="C34" s="17" t="str">
-        <x:v>晶圆减薄机</x:v>
-      </x:c>
-      <x:c r="D34" s="11" t="str">
-        <x:v>Wafer thinning equipment used in HBM and advanced packaging process flows.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="15" hidden="0" customHeight="1">
-      <x:c r="A35" s="10" t="str">
-        <x:v>obj_metric_tsmc_adv_packaging_capex</x:v>
-      </x:c>
-      <x:c r="B35" s="17" t="str">
-        <x:v>台积电先进封装扩产资本开支</x:v>
-      </x:c>
-      <x:c r="C35" s="17" t="str">
-        <x:v>资本开支</x:v>
-      </x:c>
-      <x:c r="D35" s="11" t="str">
-        <x:v>Capital expenditure associated with advanced packaging and CoWoS capacity expansion.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="15" hidden="0" customHeight="1">
-      <x:c r="A36" s="12" t="str">
+      <x:c r="A25" s="12" t="str">
         <x:v>obj_app_ai_server_training</x:v>
       </x:c>
-      <x:c r="B36" s="18" t="str">
+      <x:c r="B25" s="18" t="str">
         <x:v>数据中心AI训练与推理</x:v>
       </x:c>
-      <x:c r="C36" s="18" t="str">
+      <x:c r="C25" s="18" t="str">
         <x:v>数据中心计算应用</x:v>
       </x:c>
-      <x:c r="D36" s="13" t="str">
+      <x:c r="D25" s="13" t="str">
         <x:v>Demand scenario driving Blackwell GPU, HBM and advanced packaging requirements.</x:v>
       </x:c>
     </x:row>
@@ -4622,8 +3799,8 @@
     <x:col min="4" max="4" width="13.890000343322754" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="52.66999816894531" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="31.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="90.44000244140625" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="58.33000183105469" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -4757,211 +3934,29 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="10" t="str">
+      <x:c r="A6" s="12" t="str">
         <x:v>obj_company_samsung_electronics</x:v>
       </x:c>
-      <x:c r="B6" s="17" t="str">
+      <x:c r="B6" s="18" t="str">
         <x:v>三星电子</x:v>
       </x:c>
-      <x:c r="C6" s="17" t="str">
+      <x:c r="C6" s="18" t="str">
         <x:v>Samsung Electronics</x:v>
       </x:c>
-      <x:c r="D6" s="17" t="str">
+      <x:c r="D6" s="18" t="str">
         <x:v>公司</x:v>
       </x:c>
-      <x:c r="E6" s="17" t="str">
+      <x:c r="E6" s="18" t="str">
         <x:v>HBM supplier candidate.</x:v>
       </x:c>
-      <x:c r="F6" s="17" t="str">
+      <x:c r="F6" s="18" t="str">
         <x:v>Memory supplier</x:v>
       </x:c>
-      <x:c r="G6" s="17" t="str">
+      <x:c r="G6" s="18" t="str">
         <x:v>Korea</x:v>
       </x:c>
-      <x:c r="H6" s="11" t="str">
+      <x:c r="H6" s="13" t="str">
         <x:v>https://www.skhynix.com/product/hbm3e.go</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="10" t="str">
-        <x:v>obj_company_ibiden</x:v>
-      </x:c>
-      <x:c r="B7" s="17" t="str">
-        <x:v>揖斐电</x:v>
-      </x:c>
-      <x:c r="C7" s="17" t="str">
-        <x:v>Ibiden</x:v>
-      </x:c>
-      <x:c r="D7" s="17" t="str">
-        <x:v>公司</x:v>
-      </x:c>
-      <x:c r="E7" s="17" t="str">
-        <x:v>ABF substrate supplier.</x:v>
-      </x:c>
-      <x:c r="F7" s="17" t="str">
-        <x:v>IC substrate supplier</x:v>
-      </x:c>
-      <x:c r="G7" s="17" t="str">
-        <x:v>Japan</x:v>
-      </x:c>
-      <x:c r="H7" s="11" t="str">
-        <x:v>https://semiwiki.com/semiconductor-services/semiconductor-packaging/335318-understanding-tsmcs-cowos-l-packaging/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="10" t="str">
-        <x:v>obj_company_unimicron</x:v>
-      </x:c>
-      <x:c r="B8" s="17" t="str">
-        <x:v>欣兴电子</x:v>
-      </x:c>
-      <x:c r="C8" s="17" t="str">
-        <x:v>Unimicron</x:v>
-      </x:c>
-      <x:c r="D8" s="17" t="str">
-        <x:v>公司</x:v>
-      </x:c>
-      <x:c r="E8" s="17" t="str">
-        <x:v>ABF substrate supplier.</x:v>
-      </x:c>
-      <x:c r="F8" s="17" t="str">
-        <x:v>IC substrate supplier</x:v>
-      </x:c>
-      <x:c r="G8" s="17" t="str">
-        <x:v>Taiwan, China</x:v>
-      </x:c>
-      <x:c r="H8" s="11" t="str">
-        <x:v>https://semiwiki.com/semiconductor-services/semiconductor-packaging/335318-understanding-tsmcs-cowos-l-packaging/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="10" t="str">
-        <x:v>obj_company_shinko</x:v>
-      </x:c>
-      <x:c r="B9" s="17" t="str">
-        <x:v>新光电气</x:v>
-      </x:c>
-      <x:c r="C9" s="17" t="str">
-        <x:v>Shinko Electric</x:v>
-      </x:c>
-      <x:c r="D9" s="17" t="str">
-        <x:v>公司</x:v>
-      </x:c>
-      <x:c r="E9" s="17" t="str">
-        <x:v>ABF substrate supplier.</x:v>
-      </x:c>
-      <x:c r="F9" s="17" t="str">
-        <x:v>IC substrate supplier</x:v>
-      </x:c>
-      <x:c r="G9" s="17" t="str">
-        <x:v>Japan</x:v>
-      </x:c>
-      <x:c r="H9" s="11" t="str">
-        <x:v>https://semiwiki.com/semiconductor-services/semiconductor-packaging/335318-understanding-tsmcs-cowos-l-packaging/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="10" t="str">
-        <x:v>obj_company_besi</x:v>
-      </x:c>
-      <x:c r="B10" s="17" t="str">
-        <x:v>BESI</x:v>
-      </x:c>
-      <x:c r="C10" s="17" t="str">
-        <x:v>BESI</x:v>
-      </x:c>
-      <x:c r="D10" s="17" t="str">
-        <x:v>公司</x:v>
-      </x:c>
-      <x:c r="E10" s="17" t="str">
-        <x:v>Advanced bonding equipment supplier.</x:v>
-      </x:c>
-      <x:c r="F10" s="17" t="str">
-        <x:v>Semiconductor equipment supplier</x:v>
-      </x:c>
-      <x:c r="G10" s="17" t="str">
-        <x:v>Netherlands</x:v>
-      </x:c>
-      <x:c r="H10" s="11" t="str">
-        <x:v>https://semiwiki.com/semiconductor-services/semiconductor-packaging/335318-understanding-tsmcs-cowos-l-packaging/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="10" t="str">
-        <x:v>obj_company_asmpt</x:v>
-      </x:c>
-      <x:c r="B11" s="17" t="str">
-        <x:v>ASMPT</x:v>
-      </x:c>
-      <x:c r="C11" s="17" t="str">
-        <x:v>ASMPT</x:v>
-      </x:c>
-      <x:c r="D11" s="17" t="str">
-        <x:v>公司</x:v>
-      </x:c>
-      <x:c r="E11" s="17" t="str">
-        <x:v>Advanced bonding equipment supplier.</x:v>
-      </x:c>
-      <x:c r="F11" s="17" t="str">
-        <x:v>Semiconductor equipment supplier</x:v>
-      </x:c>
-      <x:c r="G11" s="17" t="str">
-        <x:v>Hong Kong, China</x:v>
-      </x:c>
-      <x:c r="H11" s="11" t="str">
-        <x:v>https://semiwiki.com/semiconductor-services/semiconductor-packaging/335318-understanding-tsmcs-cowos-l-packaging/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="10" t="str">
-        <x:v>obj_company_kulicke_soffa</x:v>
-      </x:c>
-      <x:c r="B12" s="17" t="str">
-        <x:v>K&amp;S</x:v>
-      </x:c>
-      <x:c r="C12" s="17" t="str">
-        <x:v>Kulicke &amp; Soffa</x:v>
-      </x:c>
-      <x:c r="D12" s="17" t="str">
-        <x:v>公司</x:v>
-      </x:c>
-      <x:c r="E12" s="17" t="str">
-        <x:v>Bonding equipment supplier.</x:v>
-      </x:c>
-      <x:c r="F12" s="17" t="str">
-        <x:v>Semiconductor equipment supplier</x:v>
-      </x:c>
-      <x:c r="G12" s="17" t="str">
-        <x:v>United States</x:v>
-      </x:c>
-      <x:c r="H12" s="11" t="str">
-        <x:v>https://semiwiki.com/semiconductor-services/semiconductor-packaging/335318-understanding-tsmcs-cowos-l-packaging/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="12" t="str">
-        <x:v>obj_company_disco</x:v>
-      </x:c>
-      <x:c r="B13" s="18" t="str">
-        <x:v>DISCO</x:v>
-      </x:c>
-      <x:c r="C13" s="18" t="str">
-        <x:v>DISCO</x:v>
-      </x:c>
-      <x:c r="D13" s="18" t="str">
-        <x:v>公司</x:v>
-      </x:c>
-      <x:c r="E13" s="18" t="str">
-        <x:v>Wafer thinning and dicing equipment supplier.</x:v>
-      </x:c>
-      <x:c r="F13" s="18" t="str">
-        <x:v>Semiconductor equipment supplier</x:v>
-      </x:c>
-      <x:c r="G13" s="18" t="str">
-        <x:v>Japan</x:v>
-      </x:c>
-      <x:c r="H13" s="13" t="str">
-        <x:v>https://semiwiki.com/semiconductor-services/semiconductor-packaging/335318-understanding-tsmcs-cowos-l-packaging/</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>